<commit_message>
Migrate CHIP "What is CHIP?" page
Add /western-pennsylvania/chip/what-is-chip to the existing chip template
and style its FAQ accordion inside the CHIP article layout.

Import:
- chip template: add the what-is-chip URL and an accordion-minimal-light
  block (reuses the sidebar-FAQ parser unchanged); restore its description
- import-chip.js registers the accordion parser and embeds the updated
  template; the three existing CHIP pages re-import byte-identical

Styling (scoped to body.chip):
- accordion-minimal-light: source fonts, chevron, answer lists and link
  styling; the sidebar-page offset rules skip CHIP pages; first item opens
  by default on CHIP pages only
- styles.css: the accordion section keeps the article column width, with
  the source's 20px spacing above and 60px article padding below

Sidebar FAQ pages and the other CHIP pages render unchanged.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-chip.report.xlsx
+++ b/tools/importer/reports/import-chip.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="272">
   <si>
     <t>_reportFile</t>
   </si>
@@ -163,6 +163,27 @@
     <t>https://www.highmark.com/resources/spending-accounts</t>
   </si>
   <si>
+    <t>western-pennsylvania/chip.report.json</t>
+  </si>
+  <si>
+    <t>["hero-minimal-dark-withimg","cards-minimal-dark-iconnav","cards-minimal-dark-withimg-icons","columns-minimal-dark","cards-minimal-dark-withimg-2"]</t>
+  </si>
+  <si>
+    <t>western-pennsylvania/chip</t>
+  </si>
+  <si>
+    <t>chip-landing</t>
+  </si>
+  <si>
+    <t>2026-09-29T21:31:20.155Z</t>
+  </si>
+  <si>
+    <t>CHIP - Highmark Healthy Kids | Highmark Blue Cross Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/western-pennsylvania/chip?zg=false</t>
+  </si>
+  <si>
     <t>resources/answers/articles.report.json</t>
   </si>
   <si>
@@ -382,7 +403,7 @@
     <t>chip</t>
   </si>
   <si>
-    <t>2026-09-29T18:58:27.624Z</t>
+    <t>2026-09-29T23:06:19.341Z</t>
   </si>
   <si>
     <t>CHIP Eligibility and Costs | Highmark Blue Cross Blue Shield</t>
@@ -400,7 +421,7 @@
     <t>western-pennsylvania/chip/chip-resources</t>
   </si>
   <si>
-    <t>2026-09-29T18:58:33.743Z</t>
+    <t>2026-09-29T23:06:25.278Z</t>
   </si>
   <si>
     <t>CHIP Resources | Highmark Blue Cross Blue Shield</t>
@@ -415,13 +436,31 @@
     <t>western-pennsylvania/chip/doctors-drugs</t>
   </si>
   <si>
-    <t>2026-09-29T18:58:38.501Z</t>
+    <t>2026-09-29T23:06:30.949Z</t>
   </si>
   <si>
     <t>CHIP Doctors and Drugs | Highmark Blue Cross Blue Shield</t>
   </si>
   <si>
     <t>https://www.highmark.com/western-pennsylvania/chip/doctors-drugs?zg=false</t>
+  </si>
+  <si>
+    <t>western-pennsylvania/chip/what-is-chip.report.json</t>
+  </si>
+  <si>
+    <t>["cards-minimal-light-sidenav","accordion-minimal-light"]</t>
+  </si>
+  <si>
+    <t>western-pennsylvania/chip/what-is-chip</t>
+  </si>
+  <si>
+    <t>2026-09-29T23:06:37.905Z</t>
+  </si>
+  <si>
+    <t>What is CHIP? | Highmark Blue Cross Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/western-pennsylvania/chip/what-is-chip?zg=false</t>
   </si>
   <si>
     <t>resources/answers/articles/spending-accounts.report.json</t>
@@ -1176,7 +1215,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1398,114 +1437,114 @@
         <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="F12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -1514,24 +1553,24 @@
         <v>46</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1540,47 +1579,47 @@
         <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
         <v>99</v>
@@ -1589,27 +1628,27 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -1618,24 +1657,24 @@
         <v>33</v>
       </c>
       <c r="F17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B18" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -1644,24 +1683,24 @@
         <v>33</v>
       </c>
       <c r="F18" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G18" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H18" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -1670,30 +1709,30 @@
         <v>33</v>
       </c>
       <c r="F19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B20" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>122</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
         <v>123</v>
@@ -1719,102 +1758,102 @@
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F21" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G21" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H21" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B22" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C22" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F22" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H22" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>134</v>
       </c>
       <c r="C23" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="F23" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G23" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>53</v>
+        <v>129</v>
       </c>
       <c r="F24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G24" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H24" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B25" t="s">
-        <v>150</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
         <v>151</v>
@@ -1840,519 +1879,571 @@
         <v>156</v>
       </c>
       <c r="B26" t="s">
-        <v>63</v>
+        <v>157</v>
       </c>
       <c r="C26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>53</v>
+        <v>165</v>
       </c>
       <c r="F27" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G27" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H27" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B28" t="s">
-        <v>144</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G28" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H28" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B29" t="s">
-        <v>51</v>
+        <v>175</v>
       </c>
       <c r="C29" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F29" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="G29" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H29" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B30" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C30" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F30" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G30" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="H30" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B31" t="s">
-        <v>183</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>152</v>
+        <v>60</v>
       </c>
       <c r="F31" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G31" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H31" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B32" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="C32" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F32" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G32" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H32" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
+        <v>196</v>
       </c>
       <c r="C33" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D33" t="s">
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>53</v>
+        <v>165</v>
       </c>
       <c r="F33" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="G33" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="H33" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B34" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="C34" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F34" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="G34" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H34" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B35" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C35" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D35" t="s">
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F35" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="G35" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="H35" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B36" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="C36" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>210</v>
+        <v>60</v>
       </c>
       <c r="F36" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G36" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H36" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B37" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="C37" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>152</v>
+        <v>60</v>
       </c>
       <c r="F37" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G37" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="H37" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B38" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C38" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>53</v>
+        <v>223</v>
       </c>
       <c r="F38" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="G38" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="H38" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B39" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="C39" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>210</v>
+        <v>165</v>
       </c>
       <c r="F39" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G39" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="H39" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="C40" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="F40" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G40" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H40" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>157</v>
       </c>
       <c r="C41" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>93</v>
+        <v>223</v>
       </c>
       <c r="F41" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G41" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="H41" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B42" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C42" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F42" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="G42" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="H42" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B43" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C43" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F43" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="G43" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="H43" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B44" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C44" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="F44" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G44" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="H44" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B45" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C45" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F45" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G45" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H45" t="s">
-        <v>258</v>
+        <v>261</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>262</v>
+      </c>
+      <c r="B46" t="s">
+        <v>58</v>
+      </c>
+      <c r="C46" t="s">
+        <v>263</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>152</v>
+      </c>
+      <c r="F46" t="s">
+        <v>264</v>
+      </c>
+      <c r="G46" t="s">
+        <v>265</v>
+      </c>
+      <c r="H46" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>267</v>
+      </c>
+      <c r="B47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" t="s">
+        <v>268</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>100</v>
+      </c>
+      <c r="F47" t="s">
+        <v>269</v>
+      </c>
+      <c r="G47" t="s">
+        <v>270</v>
+      </c>
+      <c r="H47" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Migrate CHIP "What is CHIP?" page (#24)
Add /western-pennsylvania/chip/what-is-chip to the existing chip template
and style its FAQ accordion inside the CHIP article layout.

Import:
- chip template: add the what-is-chip URL and an accordion-minimal-light
  block (reuses the sidebar-FAQ parser unchanged); restore its description
- import-chip.js registers the accordion parser and embeds the updated
  template; the three existing CHIP pages re-import byte-identical

Styling (scoped to body.chip):
- accordion-minimal-light: source fonts, chevron, answer lists and link
  styling; the sidebar-page offset rules skip CHIP pages; first item opens
  by default on CHIP pages only
- styles.css: the accordion section keeps the article column width, with
  the source's 20px spacing above and 60px article padding below

Sidebar FAQ pages and the other CHIP pages render unchanged.

Co-authored-by: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-chip.report.xlsx
+++ b/tools/importer/reports/import-chip.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="272">
   <si>
     <t>_reportFile</t>
   </si>
@@ -163,6 +163,27 @@
     <t>https://www.highmark.com/resources/spending-accounts</t>
   </si>
   <si>
+    <t>western-pennsylvania/chip.report.json</t>
+  </si>
+  <si>
+    <t>["hero-minimal-dark-withimg","cards-minimal-dark-iconnav","cards-minimal-dark-withimg-icons","columns-minimal-dark","cards-minimal-dark-withimg-2"]</t>
+  </si>
+  <si>
+    <t>western-pennsylvania/chip</t>
+  </si>
+  <si>
+    <t>chip-landing</t>
+  </si>
+  <si>
+    <t>2026-09-29T21:31:20.155Z</t>
+  </si>
+  <si>
+    <t>CHIP - Highmark Healthy Kids | Highmark Blue Cross Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/western-pennsylvania/chip?zg=false</t>
+  </si>
+  <si>
     <t>resources/answers/articles.report.json</t>
   </si>
   <si>
@@ -382,7 +403,7 @@
     <t>chip</t>
   </si>
   <si>
-    <t>2026-09-29T18:58:27.624Z</t>
+    <t>2026-09-29T23:06:19.341Z</t>
   </si>
   <si>
     <t>CHIP Eligibility and Costs | Highmark Blue Cross Blue Shield</t>
@@ -400,7 +421,7 @@
     <t>western-pennsylvania/chip/chip-resources</t>
   </si>
   <si>
-    <t>2026-09-29T18:58:33.743Z</t>
+    <t>2026-09-29T23:06:25.278Z</t>
   </si>
   <si>
     <t>CHIP Resources | Highmark Blue Cross Blue Shield</t>
@@ -415,13 +436,31 @@
     <t>western-pennsylvania/chip/doctors-drugs</t>
   </si>
   <si>
-    <t>2026-09-29T18:58:38.501Z</t>
+    <t>2026-09-29T23:06:30.949Z</t>
   </si>
   <si>
     <t>CHIP Doctors and Drugs | Highmark Blue Cross Blue Shield</t>
   </si>
   <si>
     <t>https://www.highmark.com/western-pennsylvania/chip/doctors-drugs?zg=false</t>
+  </si>
+  <si>
+    <t>western-pennsylvania/chip/what-is-chip.report.json</t>
+  </si>
+  <si>
+    <t>["cards-minimal-light-sidenav","accordion-minimal-light"]</t>
+  </si>
+  <si>
+    <t>western-pennsylvania/chip/what-is-chip</t>
+  </si>
+  <si>
+    <t>2026-09-29T23:06:37.905Z</t>
+  </si>
+  <si>
+    <t>What is CHIP? | Highmark Blue Cross Blue Shield</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/western-pennsylvania/chip/what-is-chip?zg=false</t>
   </si>
   <si>
     <t>resources/answers/articles/spending-accounts.report.json</t>
@@ -1176,7 +1215,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1398,114 +1437,114 @@
         <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="F12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -1514,24 +1553,24 @@
         <v>46</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1540,47 +1579,47 @@
         <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>93</v>
+        <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
         <v>99</v>
@@ -1589,27 +1628,27 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -1618,24 +1657,24 @@
         <v>33</v>
       </c>
       <c r="F17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B18" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
@@ -1644,24 +1683,24 @@
         <v>33</v>
       </c>
       <c r="F18" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G18" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H18" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
@@ -1670,30 +1709,30 @@
         <v>33</v>
       </c>
       <c r="F19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B20" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>122</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
         <v>123</v>
@@ -1719,102 +1758,102 @@
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F21" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G21" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H21" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B22" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C22" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F22" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H22" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>134</v>
       </c>
       <c r="C23" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="F23" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G23" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>53</v>
+        <v>129</v>
       </c>
       <c r="F24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G24" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H24" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B25" t="s">
-        <v>150</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
         <v>151</v>
@@ -1840,519 +1879,571 @@
         <v>156</v>
       </c>
       <c r="B26" t="s">
-        <v>63</v>
+        <v>157</v>
       </c>
       <c r="C26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>53</v>
+        <v>165</v>
       </c>
       <c r="F27" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G27" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H27" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B28" t="s">
-        <v>144</v>
+        <v>70</v>
       </c>
       <c r="C28" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G28" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H28" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B29" t="s">
-        <v>51</v>
+        <v>175</v>
       </c>
       <c r="C29" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F29" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="G29" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H29" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B30" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C30" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F30" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="G30" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="H30" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B31" t="s">
-        <v>183</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>152</v>
+        <v>60</v>
       </c>
       <c r="F31" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G31" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H31" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B32" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="C32" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F32" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G32" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H32" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
+        <v>196</v>
       </c>
       <c r="C33" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D33" t="s">
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>53</v>
+        <v>165</v>
       </c>
       <c r="F33" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="G33" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="H33" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B34" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="C34" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F34" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="G34" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H34" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B35" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C35" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D35" t="s">
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F35" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="G35" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="H35" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B36" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="C36" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>210</v>
+        <v>60</v>
       </c>
       <c r="F36" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G36" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H36" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B37" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="C37" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>152</v>
+        <v>60</v>
       </c>
       <c r="F37" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G37" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="H37" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B38" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C38" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>53</v>
+        <v>223</v>
       </c>
       <c r="F38" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="G38" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="H38" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B39" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="C39" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>210</v>
+        <v>165</v>
       </c>
       <c r="F39" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G39" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="H39" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="C40" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="F40" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G40" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="H40" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>157</v>
       </c>
       <c r="C41" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>93</v>
+        <v>223</v>
       </c>
       <c r="F41" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G41" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="H41" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B42" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C42" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F42" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="G42" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="H42" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B43" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C43" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F43" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="G43" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="H43" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B44" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C44" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="F44" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G44" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="H44" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B45" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C45" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F45" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G45" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H45" t="s">
-        <v>258</v>
+        <v>261</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>262</v>
+      </c>
+      <c r="B46" t="s">
+        <v>58</v>
+      </c>
+      <c r="C46" t="s">
+        <v>263</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>152</v>
+      </c>
+      <c r="F46" t="s">
+        <v>264</v>
+      </c>
+      <c r="G46" t="s">
+        <v>265</v>
+      </c>
+      <c r="H46" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>267</v>
+      </c>
+      <c r="B47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" t="s">
+        <v>268</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>100</v>
+      </c>
+      <c r="F47" t="s">
+        <v>269</v>
+      </c>
+      <c r="G47" t="s">
+        <v>270</v>
+      </c>
+      <c r="H47" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>